<commit_message>
Update sample Excel and CSV question download templates to function-based LeetCode style format
</commit_message>
<xml_diff>
--- a/frontend/public/sample_questions_template.xlsx
+++ b/frontend/public/sample_questions_template.xlsx
@@ -490,17 +490,14 @@
         <v>Array, Hash Table</v>
       </c>
       <c r="E2" t="str" xml:space="preserve">
-        <v xml:space="preserve">Given an array of integers nums and an integer target, return indices of the two numbers such that they add up to target. You may assume that each input would have exactly one solution, and you may not use the same element twice.
-Input:
-First line contains integer N (size of array)
-Second line contains N integers
-Third line contains integer target</v>
+        <v xml:space="preserve">Given an array of integers nums and an integer target, return indices of the two numbers such that they add up to target.
+You may assume that each input would have exactly one solution, and you may not use the same element twice. Return the answer as an integer array of two indices.</v>
       </c>
       <c r="F2" t="str">
-        <v>N on line 1, array elements on line 2, target on line 3</v>
+        <v>[nums] on line 1, target on line 2 (or N on line 1, array elements on line 2, target on line 3)</v>
       </c>
       <c r="G2" t="str">
-        <v>Two indices separated by space</v>
+        <v>[index1, index2]</v>
       </c>
       <c r="H2" t="str" xml:space="preserve">
         <v xml:space="preserve">2 &lt;= nums.length &lt;= 10^4
@@ -509,80 +506,70 @@
       </c>
       <c r="I2" t="str" xml:space="preserve">
         <v xml:space="preserve">import java.util.*;
-public class Main {
-    public static void main(String[] args) {
-        Scanner sc = new Scanner(System.in);
-        int n = sc.nextInt();
-        int[] nums = new int[n];
-        for(int i = 0; i &lt; n; i++) nums[i] = sc.nextInt();
-        int target = sc.nextInt();
+class Solution {
+    public int[] twoSum(int[] nums, int target) {
         // Write your solution here
         Map&lt;Integer, Integer&gt; map = new HashMap&lt;&gt;();
-        for(int i = 0; i &lt; n; i++) {
+        for (int i = 0; i &lt; nums.length; i++) {
             int complement = target - nums[i];
-            if(map.containsKey(complement)) {
-                System.out.println(map.get(complement) + " " + i);
-                return;
+            if (map.containsKey(complement)) {
+                return new int[] { map.get(complement), i };
             }
             map.put(nums[i], i);
         }
+        return new int[]{};
     }
 }</v>
       </c>
       <c r="J2" t="str">
-        <v>Use a HashMap to store the numbers you have seen so far for O(N) time complexity.</v>
+        <v>Use a HashMap to store values and their indices for O(N) lookup.</v>
       </c>
       <c r="K2" t="str" xml:space="preserve">
-        <v xml:space="preserve">4
-2 7 11 15
+        <v xml:space="preserve">[2, 7, 11, 15]
 9</v>
       </c>
       <c r="L2" t="str">
-        <v>0 1</v>
+        <v>[0, 1]</v>
       </c>
       <c r="M2" t="str">
-        <v>nums[0] + nums[1] == 9, we return 0 1.</v>
+        <v>Because nums[0] + nums[1] == 9, we return [0, 1].</v>
       </c>
       <c r="N2" t="str" xml:space="preserve">
-        <v xml:space="preserve">3
-3 2 4
+        <v xml:space="preserve">[3, 2, 4]
 6</v>
       </c>
       <c r="O2" t="str">
-        <v>1 2</v>
+        <v>[1, 2]</v>
       </c>
       <c r="P2" t="str">
-        <v>nums[1] + nums[2] == 6, we return 1 2.</v>
+        <v>Because nums[1] + nums[2] == 6, we return [1, 2].</v>
       </c>
       <c r="Q2" t="str" xml:space="preserve">
-        <v xml:space="preserve">4
-2 7 11 15
+        <v xml:space="preserve">[2, 7, 11, 15]
 9</v>
       </c>
       <c r="R2" t="str">
-        <v>0 1</v>
+        <v>[0, 1]</v>
       </c>
       <c r="S2" t="str">
         <v>FALSE</v>
       </c>
       <c r="T2" t="str" xml:space="preserve">
-        <v xml:space="preserve">3
-3 2 4
+        <v xml:space="preserve">[3, 2, 4]
 6</v>
       </c>
       <c r="U2" t="str">
-        <v>1 2</v>
+        <v>[1, 2]</v>
       </c>
       <c r="V2" t="str">
         <v>FALSE</v>
       </c>
       <c r="W2" t="str" xml:space="preserve">
-        <v xml:space="preserve">2
-3 3
+        <v xml:space="preserve">[3, 3]
 6</v>
       </c>
       <c r="X2" t="str">
-        <v>0 1</v>
+        <v>[0, 1]</v>
       </c>
       <c r="Y2" t="str">
         <v>TRUE</v>
@@ -590,85 +577,90 @@
     </row>
     <row r="3" xml:space="preserve">
       <c r="A3" t="str">
-        <v>Reverse a String</v>
+        <v>Valid Parentheses</v>
       </c>
       <c r="B3" t="str">
-        <v>Strings</v>
+        <v>Stacks</v>
       </c>
       <c r="C3" t="str">
         <v>Easy</v>
       </c>
       <c r="D3" t="str">
-        <v>String, Two Pointers</v>
-      </c>
-      <c r="E3" t="str">
-        <v>Write a Java program that takes a string as input and prints the reversed string.</v>
+        <v>String, Stack</v>
+      </c>
+      <c r="E3" t="str" xml:space="preserve">
+        <v xml:space="preserve">Given a string s containing just the characters '(', ')', '{', '}', '[' and ']', determine if the input string is valid.
+An input string is valid if open brackets are closed by the same type of brackets and in the correct order.</v>
       </c>
       <c r="F3" t="str">
-        <v>A single line containing string S</v>
+        <v>A single string s</v>
       </c>
       <c r="G3" t="str">
-        <v>Reversed string</v>
+        <v>true or false</v>
       </c>
       <c r="H3" t="str">
-        <v>1 &lt;= S.length &lt;= 10^5</v>
+        <v>1 &lt;= s.length &lt;= 10^4</v>
       </c>
       <c r="I3" t="str" xml:space="preserve">
         <v xml:space="preserve">import java.util.*;
-public class Main {
-    public static void main(String[] args) {
-        Scanner sc = new Scanner(System.in);
-        String s = sc.nextLine();
-        // Reverse and print
-        StringBuilder sb = new StringBuilder(s);
-        System.out.println(sb.reverse().toString());
+class Solution {
+    public boolean isValid(String s) {
+        // Write your solution here
+        Stack&lt;Character&gt; stack = new Stack&lt;&gt;();
+        for (char c : s.toCharArray()) {
+            if (c == '(') stack.push(')');
+            else if (c == '{') stack.push('}');
+            else if (c == '[') stack.push(']');
+            else if (stack.isEmpty() || stack.pop() != c) return false;
+        }
+        return stack.isEmpty();
     }
 }</v>
       </c>
       <c r="J3" t="str">
-        <v>You can use StringBuilder.reverse() or two pointers.</v>
+        <v>Use a Stack to push expected closing brackets when an opening bracket is encountered.</v>
       </c>
       <c r="K3" t="str">
-        <v>hello</v>
+        <v>"()"</v>
       </c>
       <c r="L3" t="str">
-        <v>olleh</v>
+        <v>true</v>
       </c>
       <c r="M3" t="str">
-        <v>The reverse of hello is olleh.</v>
+        <v>The brackets open and close properly.</v>
       </c>
       <c r="N3" t="str">
-        <v>Java</v>
+        <v>"()[]{}"</v>
       </c>
       <c r="O3" t="str">
-        <v>avaJ</v>
+        <v>true</v>
       </c>
       <c r="P3" t="str">
-        <v>The reverse of Java is avaJ.</v>
+        <v>All bracket types are closed in correct order.</v>
       </c>
       <c r="Q3" t="str">
-        <v>hello</v>
+        <v>"()"</v>
       </c>
       <c r="R3" t="str">
-        <v>olleh</v>
+        <v>true</v>
       </c>
       <c r="S3" t="str">
         <v>FALSE</v>
       </c>
       <c r="T3" t="str">
-        <v>Java</v>
+        <v>"()[]{}"</v>
       </c>
       <c r="U3" t="str">
-        <v>avaJ</v>
+        <v>true</v>
       </c>
       <c r="V3" t="str">
         <v>FALSE</v>
       </c>
       <c r="W3" t="str">
-        <v>DSA Practice Platform</v>
+        <v>"(]"</v>
       </c>
       <c r="X3" t="str">
-        <v>mroftalP ecitcarP ASD</v>
+        <v>false</v>
       </c>
       <c r="Y3" t="str">
         <v>TRUE</v>

</xml_diff>